<commit_message>
Add new UI elements and localization support
- Created a new prefab for Key 1 in the Global Prefabs directory.
- Implemented DeselectOnPointerExit script to handle UI deselection on pointer exit in the Title Scene.
- Added back button hover and default images for the Title Scene.
- Included title left hover and default images for the Title Scene.
- Introduced localization support with a new strings.xlsx file for text management.
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Localization/strings.xlsx
+++ b/Assets/StreamingAssets/Localization/strings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\FYP\Assets\StreamingAssets\Localization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C103866C-6057-410A-B062-C64A954E0B6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC1D4928-B9B9-4C59-B6EC-62C7A1345CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3408" yWindow="2268" windowWidth="19032" windowHeight="8832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="16080" windowHeight="11028" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1-Scene-1" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="132">
   <si>
     <t>zh</t>
   </si>
@@ -107,9 +107,6 @@
     <t>Key Bindings</t>
   </si>
   <si>
-    <t>Speed</t>
-  </si>
-  <si>
     <t>文本速率</t>
   </si>
   <si>
@@ -411,6 +408,30 @@
   </si>
   <si>
     <t>· this trip was really thrilling; I almost ran right into the director on the fifth floor. I decide to wedge the iron door with a stone—if the wind blows it shut, it’s over.</t>
+  </si>
+  <si>
+    <t>进入游戏</t>
+  </si>
+  <si>
+    <t>Enter Game</t>
+  </si>
+  <si>
+    <t>退出游戏</t>
+  </si>
+  <si>
+    <t>Exit Game</t>
+  </si>
+  <si>
+    <t>Run Speed</t>
+  </si>
+  <si>
+    <t>Move Speed</t>
+  </si>
+  <si>
+    <t>返回标题</t>
+  </si>
+  <si>
+    <t>Back</t>
   </si>
 </sst>
 </file>
@@ -731,7 +752,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5125BF64-7B82-433D-8FED-955690D00D20}">
-  <dimension ref="A1:B64"/>
+  <dimension ref="A1:B67"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="80.44140625" customWidth="1"/>
@@ -748,10 +769,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" t="s">
         <v>98</v>
-      </c>
-      <c r="B2" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -759,7 +780,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -823,7 +844,7 @@
         <v>17</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>23</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -831,7 +852,7 @@
         <v>18</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>9</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -850,404 +871,428 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B42" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B43" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B44" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B45" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B46" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B47" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B48" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B50" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B51" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B52" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B53" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B54" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B55" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B56" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B57" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B58" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B59" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B60" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B61" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
+        <v>106</v>
+      </c>
+      <c r="B62" t="s">
         <v>107</v>
-      </c>
-      <c r="B62" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
+        <v>109</v>
+      </c>
+      <c r="B63" t="s">
         <v>110</v>
-      </c>
-      <c r="B63" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B64" t="s">
-        <v>119</v>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>124</v>
+      </c>
+      <c r="B65" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>126</v>
+      </c>
+      <c r="B66" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>130</v>
+      </c>
+      <c r="B67" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add metadata for new ICON.png asset in Global Sprites directory
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Localization/strings.xlsx
+++ b/Assets/StreamingAssets/Localization/strings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\FYP\Assets\StreamingAssets\Localization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCC1E92-3D7B-4A70-B733-A5FA78E82DCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B445D2E-90BD-4F57-BCC3-0D6C68D20C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="936" yWindow="2088" windowWidth="16080" windowHeight="11028" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="936" yWindow="1212" windowWidth="16080" windowHeight="11028" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1-Scene-1" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="146">
   <si>
     <t>zh</t>
   </si>
@@ -470,6 +470,12 @@
   <si>
     <t>Are you sure you want to quit the game and return to the title screen? Your current progress will be lost.
 Tip: If you only want to close the pause menu, press ESC again to resume the game.</t>
+  </si>
+  <si>
+    <t>结束</t>
+  </si>
+  <si>
+    <t>End</t>
   </si>
 </sst>
 </file>
@@ -790,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5125BF64-7B82-433D-8FED-955690D00D20}">
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="80.44140625" customWidth="1"/>
@@ -1379,6 +1385,14 @@
       </c>
       <c r="B73" s="1" t="s">
         <v>143</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>144</v>
+      </c>
+      <c r="B74" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add localization files for 2-Scene-UI
- Created new strings.json.meta file for localization.
- Added strings.xlsx file containing localization strings.
- Created corresponding meta file for strings.xlsx.
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Localization/strings.xlsx
+++ b/Assets/StreamingAssets/Localization/strings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\FYP\Assets\StreamingAssets\Localization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B445D2E-90BD-4F57-BCC3-0D6C68D20C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F54A8500-A0F0-4E8E-87E5-C4D44C49C2F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="936" yWindow="1212" windowWidth="16080" windowHeight="11028" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="154">
   <si>
     <t>zh</t>
   </si>
@@ -464,18 +464,40 @@
     <t>Chapter 2</t>
   </si>
   <si>
-    <t>确定要退出游戏并返回标题界面吗？当前游戏进度将会丢失。
-提示：若您只是想关闭暂停菜单，再按一次 ESC 即可返回游戏</t>
-  </si>
-  <si>
-    <t>Are you sure you want to quit the game and return to the title screen? Your current progress will be lost.
-Tip: If you only want to close the pause menu, press ESC again to resume the game.</t>
-  </si>
-  <si>
     <t>结束</t>
   </si>
   <si>
     <t>End</t>
+  </si>
+  <si>
+    <t>This chapter is currently in development and is not yet available to play.</t>
+  </si>
+  <si>
+    <t>本章正在制作中，暂未开放游玩</t>
+  </si>
+  <si>
+    <t>继续游玩</t>
+  </si>
+  <si>
+    <t>Continue</t>
+  </si>
+  <si>
+    <t>本章进度已保存\n建议直接&lt;color=#FFC600&gt;继续游玩&lt;/color&gt;，以保持剧情体验的连贯性\n若选择&lt;color=#FFC600&gt;返回标题&lt;/color&gt;，请注意：当前存档系统仍在完善中，部分功能（如日记、背包）在下次游玩时，可能出现数据不同步的情况</t>
+  </si>
+  <si>
+    <t>Your progress in this chapter has been saved.\nWe recommend selecting &lt;color=#FFC600&gt;Continue&lt;/color&gt; to keep the story experience smooth and uninterrupted. \nIf you choose &lt;color=#FFC600&gt;Back&lt;/color&gt; to Title, please note that the save system is still being improved, and some features (such as the Diary and Inventory) may not sync correctly the next time you play.</t>
+  </si>
+  <si>
+    <t>Are you sure you want to quit the game and return to the title screen? Your current progress will be lost.\n\nTip: If you only want to close the pause menu, press ESC again to resume the game.</t>
+  </si>
+  <si>
+    <t>确认</t>
+  </si>
+  <si>
+    <t>Confirm</t>
+  </si>
+  <si>
+    <t>确定要退出游戏并返回标题界面吗？当前游戏进度将会丢失\n\n提示：若您只是想关闭暂停菜单，再按一次 ESC 即可返回游戏</t>
   </si>
 </sst>
 </file>
@@ -796,7 +818,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5125BF64-7B82-433D-8FED-955690D00D20}">
-  <dimension ref="A1:B74"/>
+  <dimension ref="A1:B78"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="80.44140625" customWidth="1"/>
@@ -1379,20 +1401,52 @@
         <v>141</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
+        <v>142</v>
+      </c>
+      <c r="B74" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>145</v>
+      </c>
+      <c r="B75" t="s">
         <v>144</v>
       </c>
-      <c r="B74" t="s">
-        <v>145</v>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>146</v>
+      </c>
+      <c r="B76" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A77" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>151</v>
+      </c>
+      <c r="B78" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>